<commit_message>
Tech stack and teams
</commit_message>
<xml_diff>
--- a/Project Teams Final.xlsx
+++ b/Project Teams Final.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nikhi\OneDrive\Desktop\mern_blr\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{937D6CAD-2D7D-4DA1-A539-70E7C24DCF36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64A37111-6FCC-4E4E-BBF6-577DE0A19513}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{A37301D1-B243-43D2-8D20-1790E0FF8940}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" activeTab="1" xr2:uid="{A37301D1-B243-43D2-8D20-1790E0FF8940}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Teams" sheetId="1" r:id="rId1"/>
+    <sheet name="Tech stack" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="35">
   <si>
     <t xml:space="preserve">Karthik </t>
   </si>
@@ -132,6 +133,15 @@
   </si>
   <si>
     <t>Leader</t>
+  </si>
+  <si>
+    <t>front end - react</t>
+  </si>
+  <si>
+    <t>middleware - spring boot java / (node / express)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">back end - rdbms / NoSQL </t>
   </si>
 </sst>
 </file>
@@ -673,4 +683,29 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A45B7D59-412C-4D36-A4E8-0468D8765A88}">
+  <dimension ref="A1:A3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>